<commit_message>
IT WORKS now just need to add commments and make it as an .exe file
</commit_message>
<xml_diff>
--- a/Cleaned Up Forms/Reimbursement Data.xlsx
+++ b/Cleaned Up Forms/Reimbursement Data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,8 +461,10 @@
           <t>Test Jensen</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -476,284 +478,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>The Test Jensen</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>SWTM-2088_Atlassian-Git-Cheatsheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Test Jensen102220231</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Test Jensen102220231</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Test Jensen102220231</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Test Jensen</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>to test you</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Test Jensen102220231</t>
+          <t>Test Jensen102820231</t>
         </is>
       </c>
     </row>

</xml_diff>